<commit_message>
Add collapsible doc header info
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/06-FRM-600/FRM-602_Gage_Verification_Log.xlsx
+++ b/04-Bieu-Mau/06-FRM-600/FRM-602_Gage_Verification_Log.xlsx
@@ -10851,9 +10851,9 @@
   <mergeCells count="189">
     <mergeCell ref="AP27:AS27"/>
     <mergeCell ref="AH26:AK26"/>
+    <mergeCell ref="AA18:AG18"/>
+    <mergeCell ref="AL17:AO17"/>
     <mergeCell ref="AW2:BD2"/>
-    <mergeCell ref="AL17:AO17"/>
-    <mergeCell ref="AA18:AG18"/>
     <mergeCell ref="D19:H19"/>
     <mergeCell ref="AP17:AS17"/>
     <mergeCell ref="A21:C21"/>

</xml_diff>